<commit_message>
Set cost model team to 2 usta, 3 çırak, engineer, owner
Update maliyet/kâr sheet, contract personnel clause, checklist and
next-steps for the şahıs şirketi headcount.

Co-authored-by: barsokrr <barsokrr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/metraj/taseron_paket/Taseron_Saha_Hakedis_Maliyet_Paket.xlsx
+++ b/metraj/taseron_paket/Taseron_Saha_Hakedis_Maliyet_Paket.xlsx
@@ -22,8 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="12">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,6 +88,11 @@
       <b val="1"/>
       <color rgb="001F4E79"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -138,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -164,6 +171,12 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -529,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -550,7 +563,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -631,126 +643,130 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Fatura</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>İşçilik + sigorta yansıtması dahil tam hakediş faturası</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ekip</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2 usta + 3 çırak + 1 mühendis + şirket sahibi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>KDV</t>
+          <t>Fatura</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Yapım işi — %20 KDV, 4/10 tevkifat</t>
+          <t>İşçilik + sigorta yansıtması dahil tam hakediş faturası</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>KDV</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Yapım işi — %20 KDV, 4/10 tevkifat</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
           <t>YASAK</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Müteahhitte sigortalı işçi + şahıs şirketine fatura (muvazaa) YOK</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>DOSYA İÇERİĞİ</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>1) KAPAK — model ve NACE özeti</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2) HAKEDİŞ KIRIK 450 — tevkifatlı taşeron hakediş</t>
+          <t>1) KAPAK — model ve NACE özeti</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3) HAKEDİŞ DUZ 750 — tevkifatlı alternatif</t>
+          <t>2) HAKEDİŞ KIRIK 450 — tevkifatlı taşeron hakediş</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4) KIYAS — iki yöntem karşılaştırma</t>
+          <t>3) HAKEDİŞ DUZ 750 — tevkifatlı alternatif</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5) MALIYET KAR — şahıs şirketi gider/kâr/vergi simülasyonu</t>
+          <t>4) KIYAS — iki yöntem karşılaştırma</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6) UYUM CHECKLIST — SGK/İSG/vergi kontrol listesi</t>
+          <t>5) MALIYET KAR — şahıs şirketi gider/kâr/vergi simülasyonu</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>6b) HAKEDIS DONEM — dönemsel hakediş şablonu (formül tevkifatlı)</t>
+          <t>6) UYUM CHECKLIST — SGK/İSG/vergi kontrol listesi</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7) sozlesme_taslagi.md — taşeronluk sözleşmesi taslağı (Seçenek A)</t>
+          <t>6b) HAKEDIS DONEM — dönemsel hakediş şablonu (formül tevkifatlı)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>7) sozlesme_taslagi.md — taşeronluk sözleşmesi taslağı (Seçenek A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>8) SONRAKI_ADIMLAR.md — kurulum / sözleşme / saha / vergi yol haritası</t>
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>UYARI: Bu paket taslak/şablon niteliğindedir; avukat-mali müşavir-İSG uzmanı kontrolü olmadan imzalanmamalıdır.</t>
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
@@ -1802,53 +1818,77 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>ŞAHIS ŞİRKETİ — MALİYET / KÂR / VERGİ SİMÜLASYONU</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>Varsayımsal; mali müşavir ile kesinleştiriniz. Ana senaryo: Kırık 450 tevkifatlı tahsilat.</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ekip: 2 usta + 3 çırak + 1 mühendis + şirket sahibi | Ana senaryo: Kırık 450 tevkifatlı | Varsayımlar düzenlenebilir — MM teyidi şart</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>A) GİDER VARSAYIMLARI (DÜZENLENEBİLİR)</t>
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>A) EKİP YAPISI VE ÜCRET VARSAYIMLARI (DÜZENLENEBİLİR)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Gider kalemi</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Değer</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Birim</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>Rol</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Adet</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>SGK statü</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>Brüt ücret / ay (TL)</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Aylık brüt toplam</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>Süre (ay)</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>Dönem brüt toplam</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
         <is>
           <t>Not</t>
         </is>
@@ -1857,431 +1897,745 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>İşçi adedi</t>
+          <t>Usta (kalıp)</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>kişi</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Şahıs şirketi 4A sigortalı</t>
+          <t>4A — şahıs şirketi</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>55000</v>
+      </c>
+      <c r="E6" s="9">
+        <f>B6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" s="9">
+        <f>E6*F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Tecrübeli kalıp ustası</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Ortalama brüt ücret/ay</t>
+          <t>Çırak / yardımcı</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>35000</v>
+        <v>3</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>TL</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Mesai dahil kabaca</t>
+          <t>4A — şahıs şirketi</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>28000</v>
+      </c>
+      <c r="E7" s="9">
+        <f>B7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="9">
+        <f>E7*F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Asgari+ kabaca; çıraklık sözleşmesi ayrı değerlendirilebilir</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Süre</t>
+          <t>Şantiye mühendisi</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>4A — şahıs şirketi</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>65000</v>
+      </c>
+      <c r="E8" s="9">
+        <f>B8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>ay</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Kalıp işi süresi tahmini</t>
+      <c r="G8" s="9">
+        <f>E8*F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Metraj, kalite, İSG koordinasyon desteği</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>İşveren SGK+işsizlik kabaca</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>%22.5</t>
-        </is>
+          <t>Şirket sahibi</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
+          <t>4B Bağ-Kur (ücret değil)</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="9">
+        <f>B9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Maaş yazılmaz; geçim kârdan çekilir + Bağ-Kur prim</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>4A personel toplamı (adet)</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>B6+B7+B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>Aylık 4A brüt ücret toplamı</t>
+        </is>
+      </c>
+      <c r="B11" s="22">
+        <f>E6+E7+E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Dönem 4A brüt ücret toplamı</t>
+        </is>
+      </c>
+      <c r="B12" s="22">
+        <f>G6+G7+G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>B) DİĞER GİDER VARSAYIMLARI (DÜZENLENEBİLİR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Gider kalemi</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Değer</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>Birim</t>
+        </is>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>İşveren SGK+işsizlik oranı</t>
+        </is>
+      </c>
+      <c r="B16" s="26" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
           <t>oran</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Mali müşavir netleştirir</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Bağ-Kur (şahıs) aylık</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Kabaca; teşvik/indirim MM ile netleşir</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Bağ-Kur (şirket sahibi) aylık</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
         <v>10000</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>4B prim</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>4B prim — sahip için</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Muhasebe aylık</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B18" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Beyanname+defter</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>İSG/eğitim/MYB toplam</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>80000</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Çok tehlikeli sınıf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Küçük sarf</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>150000</v>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Kalıp malzemesi hariç</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Diğer (ulaşım, iletişim vb.)</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>100000</v>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>B) GELİR — GİDER — KÂR (KIRIK 450 SENARYOSU)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Kalem</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Tutar TL</t>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Beyanname + defter</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Hakediş matrahı (gelir)</t>
+          <t>İSG / eğitim / MYB toplam</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>5298030</v>
+        <v>80000</v>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Çok tehlikeli sınıf — dönem toplamı</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Fatura tahsil (matrah+6/10 KDV)</t>
+          <t>Küçük sarf (malzeme hariç)</t>
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>5933793.6</v>
+        <v>100000</v>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Ekip küçüldüğü için düşürüldü</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Ücretler toplamı</t>
+          <t>Ulaşım / iletişim / diğer</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>2520000</v>
+        <v>80000</v>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Dönem toplamı</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t>Sahip aylık geçim çekimi (opsiyonel)</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Kârdan çekim; vergi matrahını etkiler — MM ile</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Süre (ay) — referans</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>C) GELİR — GİDER — KÂR (KIRIK 450 SENARYOSU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>Kalem</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Tutar TL</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>Hesap</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Hakediş matrahı (gelir)</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>5298030</v>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Kırık 11.773,4 × 450</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Fatura tahsil (matrah+6/10 KDV)</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="n">
+        <v>5933793.6</v>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Tahsilat referansı</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>4A ücretler toplamı</t>
+        </is>
+      </c>
+      <c r="B29" s="9">
+        <f>B12</f>
+        <v/>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>2 usta + 3 çırak + 1 mühendis</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
           <t>İşveren SGK kabaca</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n">
-        <v>567000</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Bağ-Kur toplam</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="n">
-        <v>60000</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="B30" s="9">
+        <f>B29*B16</f>
+        <v/>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Ücret × SGK oranı</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Bağ-Kur toplam (sahip)</t>
+        </is>
+      </c>
+      <c r="B31" s="9">
+        <f>B17*B23</f>
+        <v/>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Aylık × süre</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Muhasebe toplam</t>
         </is>
       </c>
-      <c r="B24" s="9" t="n">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>İSG/eğitim</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="n">
-        <v>80000</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Sarf + diğer</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="n">
-        <v>250000</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>TOPLAM GİDER</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="n">
-        <v>3507000</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>TAHMİNİ TİCARİ KÂR (vergi öncesi)</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="n">
-        <v>1791030</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>C) VERGİ KABACA (Örnek dilimler — mali müşavir güncelleyecek)</t>
-        </is>
-      </c>
+      <c r="B32" s="9">
+        <f>B18*B23</f>
+        <v/>
+      </c>
+      <c r="C32" s="6" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Kalem</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Tutar TL</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Not</t>
-        </is>
-      </c>
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>İSG / eğitim / MYB</t>
+        </is>
+      </c>
+      <c r="B33" s="9">
+        <f>B19</f>
+        <v/>
+      </c>
+      <c r="C33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Tahmini Gelir Vergisi (yıllık dilimli kabaca)</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="n">
-        <v>558860.5</v>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>%15–%40 dilimler; 2026 dilimleri teyit edilmeli</t>
-        </is>
-      </c>
+          <t>Sarf + ulaşım/diğer</t>
+        </is>
+      </c>
+      <c r="B34" s="9">
+        <f>B20+B21</f>
+        <v/>
+      </c>
+      <c r="C34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
+          <t>Sahip geçim çekimi (opsiyonel)</t>
+        </is>
+      </c>
+      <c r="B35" s="9">
+        <f>B22*B23</f>
+        <v/>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Nakit çıkışı; ticari kâr hesabında ayrı gösterilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>TOPLAM İŞLETME GİDERİ (çekim hariç)</t>
+        </is>
+      </c>
+      <c r="B37" s="27">
+        <f>B29+B30+B31+B32+B33+B34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TOPLAM NAKİT ÇIKIŞI (çekim dahil)</t>
+        </is>
+      </c>
+      <c r="B38" s="22">
+        <f>B37+B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>TAHMİNİ TİCARİ KÂR (vergi öncesi, çekim hariç)</t>
+        </is>
+      </c>
+      <c r="B40" s="24">
+        <f>B27-B37</f>
+        <v/>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Matrah − işletme gideri</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Kâr sonrası sahip çekimi sonrası kalan</t>
+        </is>
+      </c>
+      <c r="B41" s="22">
+        <f>B40-B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="25" t="inlineStr">
+        <is>
+          <t>D) VERGİ KABACA (örnek — 2026 dilimleri MM ile teyit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>Kalem</t>
+        </is>
+      </c>
+      <c r="B44" s="20" t="inlineStr">
+        <is>
+          <t>Tutar TL</t>
+        </is>
+      </c>
+      <c r="C44" s="20" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Tahmini Gelir Vergisi (dilimli kabaca)</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="n">
+        <v>999752</v>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>B40 kârına göre kabaca; 2026 resmi dilimler MM ile güncellenir</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
           <t>Geçici vergi karşılığı (kabaca %15×kâr)</t>
         </is>
       </c>
-      <c r="B35" s="9" t="n">
-        <v>268654.5</v>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="B46" s="9">
+        <f>B40*0.15</f>
+        <v/>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>3’er aylık beyan; GV’den mahsup</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Damga / beyanname giderleri (yıllık kabaca)</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="n">
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Damga / beyanname (yıllık kabaca)</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Aylık damga + muhtasar vb.</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>NET KÂR (GV sonrası kabaca)</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="n">
-        <v>1220169.5</v>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>Bağ-Kur zaten giderde</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>D) DÜZ 750 İLE AYNI GİDERDE KÂR (karşılaştırma)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="28" t="inlineStr">
+        <is>
+          <t>NET KÂR (GV + damga sonrası, çekim öncesi kabaca)</t>
+        </is>
+      </c>
+      <c r="B48" s="29">
+        <f>B40-B45-B47</f>
+        <v/>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Bağ-Kur zaten giderde; sahip çekimi ayrıca</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Sahip çekimi sonrası net kalan (kabaca)</t>
+        </is>
+      </c>
+      <c r="B49" s="9">
+        <f>B48-B35</f>
+        <v/>
+      </c>
+      <c r="C49" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>E) DÜZ 750 İLE AYNI EKİP / GİDERDE KÂR</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Düz matrah</t>
         </is>
       </c>
-      <c r="B41" s="9" t="n">
+      <c r="B52" s="9" t="n">
         <v>8471775</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>Aynı toplam gider</t>
-        </is>
-      </c>
-      <c r="B42" s="9" t="n">
-        <v>3507000</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Aynı işletme gideri (çekim hariç)</t>
+        </is>
+      </c>
+      <c r="B53" s="9">
+        <f>B37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>Vergi öncesi kâr</t>
         </is>
       </c>
-      <c r="B43" s="9" t="n">
-        <v>4964775</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>UYARI: Ücret, SGK oranları, GV dilimleri ve geçici vergi hesabı 2026 güncel mevzuata göre mali müşavir tarafından revize edilmelidir. Bu sayfa karar destek simülasyonudur.</t>
+      <c r="B54" s="29">
+        <f>B52-B53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="30" t="inlineStr">
+        <is>
+          <t>UYARI: Ücret, SGK oranları, GV dilimleri ve geçici vergi 2026 güncel mevzuata göre mali müşavir tarafından revize edilmelidir. Çıraklar için çıraklık / burs / asgari ücret istisnaları ayrıca değerlendirilir. Bu sayfa karar destek simülasyonudur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="25" t="inlineStr">
+        <is>
+          <t>F) EKİP ÖZETİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Şantiye ekibi (4A)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2 usta + 3 çırak + 1 mühendis = 6 kişi</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Şirket yönetimi</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Şirket sahibi (4B Bağ-Kur) — maaşlı değil</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Toplam insan kaynağı</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>7 kişi (6 sigortalı işçi/mühendis + 1 sahip)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A46:D46"/>
+  <mergeCells count="3">
+    <mergeCell ref="A56:H56"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2293,7 +2647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2619,6 +2973,77 @@
       </c>
       <c r="D19" s="6" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>SGK</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Ekip: 2 usta + 3 çırak + 1 mühendis 4A girişleri şahıs şirketinde</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Zorunlu</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>SGK</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Şirket sahibi 4B Bağ-Kur; maaşlı 4A gibi gösterilmiyor</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Zorunlu</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>SGK</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Çıraklar için uygun sözleşme / bildirge tipi MM ile doğrulandı</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Önerilir</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>